<commit_message>
Add NDVI data per river in new Excel file
</commit_message>
<xml_diff>
--- a/basins/gee-data.xlsx
+++ b/basins/gee-data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ratrag/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2cdde6c514a5c013/Maastricht Study/Semester 1/Research Project S2/Lake Tanganyika/Lake-Tanganyika/basins/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{17F3C541-4CB7-1740-AB04-EC759EB2309D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{17F3C541-4CB7-1740-AB04-EC759EB2309D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D7941418-8FDE-C24F-BA79-16FE6BF9269C}"/>
   <bookViews>
     <workbookView xWindow="680" yWindow="660" windowWidth="28040" windowHeight="16660" xr2:uid="{BF32C6CA-295C-2C47-92BE-D3D1AED6D54F}"/>
   </bookViews>
@@ -5138,6 +5138,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:B530" xr:uid="{BA737F7F-F4DC-724A-A054-A73358CC8402}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>